<commit_message>
Updated ZAF_grids_kan model - 2025-12-11 12:26
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A41DE0F7-1B4A-4B8F-B945-BC438B151E82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B390E50-145B-487C-8B4A-EF57924035A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4159,7 +4159,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ED04ADA-17E4-4B9B-8963-E6A1ED519EC0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{841F5866-C6D2-4B33-97E1-2ABDD4225304}">
   <dimension ref="B9:H245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27313,7 +27313,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4610E5C5-390D-4D3D-A3C5-BC26EAFCF79E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B587F0BB-ED18-4FEC-909A-60D40EAC4E48}">
   <dimension ref="B9:L245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ZAF_grids_kan model - 2025-12-12 13:56
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B390E50-145B-487C-8B4A-EF57924035A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8C6E5D65-DA8B-456F-885A-8D8E63576E5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4159,7 +4159,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{841F5866-C6D2-4B33-97E1-2ABDD4225304}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46B9F38F-AB21-48D3-873F-3EFACE40E5D2}">
   <dimension ref="B9:H245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27313,7 +27313,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B587F0BB-ED18-4FEC-909A-60D40EAC4E48}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B92A12C7-4B74-4AD0-9615-673027657D35}">
   <dimension ref="B9:L245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ZAF_grids_kan model - 2026-05-25 13:05
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{798178D7-3CE3-449A-8836-909727B56FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{68444E5E-7854-47AE-8412-297D662C2BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4108,7 +4108,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BB149D8-CA8F-4B9C-907D-6FE038F6486A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{725E4E88-7490-4B8F-B4D7-E6AC2C1384AD}">
   <dimension ref="B9:H245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27334,7 +27334,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D878D5-8030-4EFA-BCE4-47E0FBF2CFA6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11909A5F-2A32-4715-AB8B-16AAB5536F1B}">
   <dimension ref="B9:L245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ZAF_grids_kan model - 2026-05-26 16:16
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{68444E5E-7854-47AE-8412-297D662C2BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C0C1BC3-DEF0-4F99-B1EE-49BCB93704A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4108,7 +4108,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{725E4E88-7490-4B8F-B4D7-E6AC2C1384AD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23C05EA4-DACE-42DA-82C5-F08A3C364498}">
   <dimension ref="B9:H245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27334,7 +27334,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11909A5F-2A32-4715-AB8B-16AAB5536F1B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{745583BE-0FD4-4ECF-A666-FBB0A7895B12}">
   <dimension ref="B9:L245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ZAF_grids_kan model - 2026-05-26 17:54
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C0C1BC3-DEF0-4F99-B1EE-49BCB93704A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2ABA65BC-AF1D-4984-B83B-B52A6BC8D425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4108,7 +4108,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23C05EA4-DACE-42DA-82C5-F08A3C364498}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F175388-9429-4F9E-A362-E0547F7A4832}">
   <dimension ref="B9:H245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27334,7 +27334,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{745583BE-0FD4-4ECF-A666-FBB0A7895B12}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2618314-D8B4-48A9-9E94-4DDD757A7306}">
   <dimension ref="B9:L245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ZAF_grids_kan model - 2026-05-27 01:11
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2ABA65BC-AF1D-4984-B83B-B52A6BC8D425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D66D83ED-8E09-4AEA-B331-25E0BAF41FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4108,7 +4108,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F175388-9429-4F9E-A362-E0547F7A4832}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C03DEF98-214F-4D0C-82DB-72CF530D17C5}">
   <dimension ref="B9:H245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27334,7 +27334,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2618314-D8B4-48A9-9E94-4DDD757A7306}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1105066-C8F1-4BEE-A78C-5CAA075F84F5}">
   <dimension ref="B9:L245"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
even lower tx cost sensi
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ZAF_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C8488D-BB10-4A28-82A9-29778EDEDB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{112678F8-7CF9-47FA-8C99-B20E600C5408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7426" uniqueCount="1156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7506" uniqueCount="1172">
   <si>
     <t>Unit</t>
   </si>
@@ -3551,6 +3551,54 @@
   </si>
   <si>
     <t>Hi.95.CF6.N.Y.2</t>
+  </si>
+  <si>
+    <t>Lo.0.CF1.Y.Y.0.1</t>
+  </si>
+  <si>
+    <t>Hi.0.CF1.Y.Y.0.1</t>
+  </si>
+  <si>
+    <t>Lo.95.CF1.Y.Y.0.1</t>
+  </si>
+  <si>
+    <t>Hi.95.CF1.Y.Y.0.1</t>
+  </si>
+  <si>
+    <t>Lo.0.CF1.N.Y.0.1</t>
+  </si>
+  <si>
+    <t>Hi.0.CF1.N.Y.0.1</t>
+  </si>
+  <si>
+    <t>Lo.95.CF1.N.Y.0.1</t>
+  </si>
+  <si>
+    <t>Hi.95.CF1.N.Y.0.1</t>
+  </si>
+  <si>
+    <t>Lo.0.CF6.Y.Y.0.1</t>
+  </si>
+  <si>
+    <t>Hi.0.CF6.Y.Y.0.1</t>
+  </si>
+  <si>
+    <t>Lo.95.CF6.Y.Y.0.1</t>
+  </si>
+  <si>
+    <t>Hi.95.CF6.Y.Y.0.1</t>
+  </si>
+  <si>
+    <t>Lo.0.CF6.N.Y.0.1</t>
+  </si>
+  <si>
+    <t>Hi.0.CF6.N.Y.0.1</t>
+  </si>
+  <si>
+    <t>Lo.95.CF6.N.Y.0.1</t>
+  </si>
+  <si>
+    <t>Hi.95.CF6.N.Y.0.1</t>
   </si>
 </sst>
 </file>
@@ -33944,7 +33992,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C50B696F-B355-4FC5-AD3E-AFDC509F717D}">
-  <dimension ref="B1:AC53"/>
+  <dimension ref="B1:AC69"/>
   <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="2.73046875" bestFit="1" customWidth="1"/>
@@ -34086,7 +34134,7 @@
         <v>tc-1.00.df-Y.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="H6" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC6,AB6:AB6)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y6:AA6)</f>
+        <f t="shared" ref="H6:H53" si="1">_xlfn.TEXTJOIN(".",TRUE,AC6,AB6:AB6)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y6:AA6)</f>
         <v>tc-1.00.df-Y.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="I6" t="str">
@@ -34105,9 +34153,9 @@
         <f>U6</f>
         <v>Y</v>
       </c>
-      <c r="M6">
-        <f t="shared" ref="M6" si="1">W6</f>
-        <v>1</v>
+      <c r="M6" t="str">
+        <f>TEXT(W6,"0.00")</f>
+        <v>1.00</v>
       </c>
       <c r="O6">
         <v>5</v>
@@ -34167,7 +34215,7 @@
         <v>tc-1.00.df-Y.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="H7" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC7,AB7:AB7)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y7:AA7)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-Y.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="I7" t="str">
@@ -34186,9 +34234,9 @@
         <f t="shared" ref="L7:L37" si="7">U7</f>
         <v>Y</v>
       </c>
-      <c r="M7">
-        <f t="shared" ref="M7:M37" si="8">W7</f>
-        <v>1</v>
+      <c r="M7" t="str">
+        <f t="shared" ref="M7:M69" si="8">TEXT(W7,"0.00")</f>
+        <v>1.00</v>
       </c>
       <c r="O7">
         <v>5</v>
@@ -34248,7 +34296,7 @@
         <v>tc-1.00.df-Y.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="H8" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC8,AB8:AB8)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y8:AA8)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-Y.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="I8" t="str">
@@ -34267,9 +34315,9 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M8">
+      <c r="M8" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O8">
         <v>5</v>
@@ -34329,7 +34377,7 @@
         <v>tc-1.00.df-Y.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="H9" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC9,AB9:AB9)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y9:AA9)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-Y.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="I9" t="str">
@@ -34348,9 +34396,9 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M9">
+      <c r="M9" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O9">
         <v>5</v>
@@ -34410,7 +34458,7 @@
         <v>tc-1.00.df-N.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="H10" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC10,AB10:AB10)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y10:AA10)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-N.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="I10" t="str">
@@ -34429,9 +34477,9 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M10">
+      <c r="M10" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O10">
         <v>5</v>
@@ -34491,7 +34539,7 @@
         <v>tc-1.00.df-N.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="H11" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC11,AB11:AB11)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y11:AA11)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-N.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="I11" t="str">
@@ -34510,9 +34558,9 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M11">
+      <c r="M11" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O11">
         <v>5</v>
@@ -34572,7 +34620,7 @@
         <v>tc-1.00.df-N.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="H12" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC12,AB12:AB12)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y12:AA12)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-N.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="I12" t="str">
@@ -34591,9 +34639,9 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M12">
+      <c r="M12" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O12">
         <v>5</v>
@@ -34653,7 +34701,7 @@
         <v>tc-1.00.df-N.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="H13" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC13,AB13:AB13)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y13:AA13)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-N.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="I13" t="str">
@@ -34672,9 +34720,9 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M13">
+      <c r="M13" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O13">
         <v>5</v>
@@ -34734,7 +34782,7 @@
         <v>tc-1.00.df-Y.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="H14" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC14,AB14:AB14)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y14:AA14)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-Y.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="I14" t="str">
@@ -34753,9 +34801,9 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M14">
+      <c r="M14" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O14">
         <v>5</v>
@@ -34815,7 +34863,7 @@
         <v>tc-1.00.df-Y.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="H15" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC15,AB15:AB15)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y15:AA15)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-Y.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="I15" t="str">
@@ -34834,9 +34882,9 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M15">
+      <c r="M15" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O15">
         <v>5</v>
@@ -34896,7 +34944,7 @@
         <v>tc-1.00.df-Y.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="H16" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC16,AB16:AB16)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y16:AA16)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-Y.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="I16" t="str">
@@ -34915,9 +34963,9 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M16">
+      <c r="M16" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O16">
         <v>5</v>
@@ -34977,7 +35025,7 @@
         <v>tc-1.00.df-Y.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="H17" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC17,AB17:AB17)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y17:AA17)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-Y.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="I17" t="str">
@@ -34996,9 +35044,9 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M17">
+      <c r="M17" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O17">
         <v>5</v>
@@ -35058,7 +35106,7 @@
         <v>tc-1.00.df-N.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="H18" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC18,AB18:AB18)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y18:AA18)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-N.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="I18" t="str">
@@ -35077,9 +35125,9 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M18">
+      <c r="M18" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O18">
         <v>5</v>
@@ -35139,7 +35187,7 @@
         <v>tc-1.00.df-N.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="H19" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC19,AB19:AB19)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y19:AA19)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-N.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="I19" t="str">
@@ -35158,9 +35206,9 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M19">
+      <c r="M19" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O19">
         <v>5</v>
@@ -35220,7 +35268,7 @@
         <v>tc-1.00.df-N.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="H20" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC20,AB20:AB20)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y20:AA20)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-N.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="I20" t="str">
@@ -35239,9 +35287,9 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M20">
+      <c r="M20" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O20">
         <v>5</v>
@@ -35301,7 +35349,7 @@
         <v>tc-1.00.df-N.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="H21" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC21,AB21:AB21)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y21:AA21)</f>
+        <f t="shared" si="1"/>
         <v>tc-1.00.df-N.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="I21" t="str">
@@ -35320,9 +35368,9 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M21">
+      <c r="M21" t="str">
         <f t="shared" si="8"/>
-        <v>1</v>
+        <v>1.00</v>
       </c>
       <c r="O21">
         <v>5</v>
@@ -35382,7 +35430,7 @@
         <v>tc-0.25.df-Y.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="H22" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC22,AB22:AB22)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y22:AA22)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-Y.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="I22" t="str">
@@ -35401,7 +35449,7 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M22">
+      <c r="M22" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -35463,7 +35511,7 @@
         <v>tc-0.25.df-Y.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="H23" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC23,AB23:AB23)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y23:AA23)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-Y.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="I23" t="str">
@@ -35482,7 +35530,7 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M23">
+      <c r="M23" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -35544,7 +35592,7 @@
         <v>tc-0.25.df-Y.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="H24" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC24,AB24:AB24)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y24:AA24)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-Y.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="I24" t="str">
@@ -35563,7 +35611,7 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M24">
+      <c r="M24" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -35625,7 +35673,7 @@
         <v>tc-0.25.df-Y.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="H25" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC25,AB25:AB25)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y25:AA25)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-Y.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="I25" t="str">
@@ -35644,7 +35692,7 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M25">
+      <c r="M25" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -35706,7 +35754,7 @@
         <v>tc-0.25.df-N.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="H26" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC26,AB26:AB26)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y26:AA26)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-N.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="I26" t="str">
@@ -35725,7 +35773,7 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M26">
+      <c r="M26" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -35787,7 +35835,7 @@
         <v>tc-0.25.df-N.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="H27" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC27,AB27:AB27)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y27:AA27)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-N.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="I27" t="str">
@@ -35806,7 +35854,7 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M27">
+      <c r="M27" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -35868,7 +35916,7 @@
         <v>tc-0.25.df-N.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="H28" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC28,AB28:AB28)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y28:AA28)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-N.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="I28" t="str">
@@ -35887,7 +35935,7 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M28">
+      <c r="M28" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -35949,7 +35997,7 @@
         <v>tc-0.25.df-N.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="H29" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC29,AB29:AB29)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y29:AA29)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-N.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="I29" t="str">
@@ -35968,7 +36016,7 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M29">
+      <c r="M29" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -36030,7 +36078,7 @@
         <v>tc-0.25.df-Y.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="H30" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC30,AB30:AB30)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y30:AA30)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-Y.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="I30" t="str">
@@ -36049,7 +36097,7 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M30">
+      <c r="M30" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -36111,7 +36159,7 @@
         <v>tc-0.25.df-Y.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="H31" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC31,AB31:AB31)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y31:AA31)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-Y.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="I31" t="str">
@@ -36130,7 +36178,7 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M31">
+      <c r="M31" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -36192,7 +36240,7 @@
         <v>tc-0.25.df-Y.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="H32" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC32,AB32:AB32)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y32:AA32)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-Y.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="I32" t="str">
@@ -36211,7 +36259,7 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M32">
+      <c r="M32" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -36273,7 +36321,7 @@
         <v>tc-0.25.df-Y.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="H33" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC33,AB33:AB33)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y33:AA33)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-Y.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="I33" t="str">
@@ -36292,7 +36340,7 @@
         <f t="shared" si="7"/>
         <v>Y</v>
       </c>
-      <c r="M33">
+      <c r="M33" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -36354,7 +36402,7 @@
         <v>tc-0.25.df-N.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="H34" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC34,AB34:AB34)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y34:AA34)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-N.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="I34" t="str">
@@ -36373,7 +36421,7 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M34">
+      <c r="M34" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -36435,7 +36483,7 @@
         <v>tc-0.25.df-N.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="H35" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC35,AB35:AB35)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y35:AA35)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-N.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="I35" t="str">
@@ -36454,7 +36502,7 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M35">
+      <c r="M35" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -36516,7 +36564,7 @@
         <v>tc-0.25.df-N.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="H36" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC36,AB36:AB36)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y36:AA36)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-N.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="I36" t="str">
@@ -36535,7 +36583,7 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M36">
+      <c r="M36" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -36597,7 +36645,7 @@
         <v>tc-0.25.df-N.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="H37" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC37,AB37:AB37)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y37:AA37)</f>
+        <f t="shared" si="1"/>
         <v>tc-0.25.df-N.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="I37" t="str">
@@ -36616,7 +36664,7 @@
         <f t="shared" si="7"/>
         <v>N</v>
       </c>
-      <c r="M37">
+      <c r="M37" t="str">
         <f t="shared" si="8"/>
         <v>0.25</v>
       </c>
@@ -36678,7 +36726,7 @@
         <v>tc-2.00.df-Y.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="H38" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC38,AB38:AB38)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y38:AA38)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-Y.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="I38" t="str">
@@ -36697,9 +36745,9 @@
         <f t="shared" ref="L38:L53" si="21">U38</f>
         <v>Y</v>
       </c>
-      <c r="M38">
-        <f t="shared" ref="M38:M53" si="22">W38</f>
-        <v>2</v>
+      <c r="M38" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O38">
         <v>5</v>
@@ -36729,7 +36777,7 @@
         <v>2</v>
       </c>
       <c r="Y38" t="str">
-        <f t="shared" ref="Y38:Y53" si="23">R$1&amp;"-"&amp;R38</f>
+        <f t="shared" ref="Y38:Y53" si="22">R$1&amp;"-"&amp;R38</f>
         <v>dm-Lo</v>
       </c>
       <c r="Z38" t="str">
@@ -36737,11 +36785,11 @@
         <v>cp-00</v>
       </c>
       <c r="AA38" t="str">
-        <f t="shared" ref="AA38:AA53" si="24">T38</f>
+        <f t="shared" ref="AA38:AA53" si="23">T38</f>
         <v>CF1</v>
       </c>
       <c r="AB38" t="str">
-        <f t="shared" ref="AB38:AB53" si="25">U$1&amp;"-"&amp;U38</f>
+        <f t="shared" ref="AB38:AB53" si="24">U$1&amp;"-"&amp;U38</f>
         <v>df-Y</v>
       </c>
       <c r="AC38" t="str">
@@ -36759,7 +36807,7 @@
         <v>tc-2.00.df-Y.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="H39" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC39,AB39:AB39)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y39:AA39)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-Y.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="I39" t="str">
@@ -36778,9 +36826,9 @@
         <f t="shared" si="21"/>
         <v>Y</v>
       </c>
-      <c r="M39">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M39" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O39">
         <v>5</v>
@@ -36810,7 +36858,7 @@
         <v>2</v>
       </c>
       <c r="Y39" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Hi</v>
       </c>
       <c r="Z39" t="str">
@@ -36818,11 +36866,11 @@
         <v>cp-00</v>
       </c>
       <c r="AA39" t="str">
+        <f t="shared" si="23"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB39" t="str">
         <f t="shared" si="24"/>
-        <v>CF1</v>
-      </c>
-      <c r="AB39" t="str">
-        <f t="shared" si="25"/>
         <v>df-Y</v>
       </c>
       <c r="AC39" t="str">
@@ -36840,7 +36888,7 @@
         <v>tc-2.00.df-Y.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="H40" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC40,AB40:AB40)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y40:AA40)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-Y.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="I40" t="str">
@@ -36859,9 +36907,9 @@
         <f t="shared" si="21"/>
         <v>Y</v>
       </c>
-      <c r="M40">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M40" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O40">
         <v>5</v>
@@ -36891,7 +36939,7 @@
         <v>2</v>
       </c>
       <c r="Y40" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Lo</v>
       </c>
       <c r="Z40" t="str">
@@ -36899,11 +36947,11 @@
         <v>cp-95</v>
       </c>
       <c r="AA40" t="str">
+        <f t="shared" si="23"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB40" t="str">
         <f t="shared" si="24"/>
-        <v>CF1</v>
-      </c>
-      <c r="AB40" t="str">
-        <f t="shared" si="25"/>
         <v>df-Y</v>
       </c>
       <c r="AC40" t="str">
@@ -36921,7 +36969,7 @@
         <v>tc-2.00.df-Y.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="H41" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC41,AB41:AB41)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y41:AA41)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-Y.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="I41" t="str">
@@ -36940,9 +36988,9 @@
         <f t="shared" si="21"/>
         <v>Y</v>
       </c>
-      <c r="M41">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M41" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O41">
         <v>5</v>
@@ -36972,7 +37020,7 @@
         <v>2</v>
       </c>
       <c r="Y41" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Hi</v>
       </c>
       <c r="Z41" t="str">
@@ -36980,11 +37028,11 @@
         <v>cp-95</v>
       </c>
       <c r="AA41" t="str">
+        <f t="shared" si="23"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB41" t="str">
         <f t="shared" si="24"/>
-        <v>CF1</v>
-      </c>
-      <c r="AB41" t="str">
-        <f t="shared" si="25"/>
         <v>df-Y</v>
       </c>
       <c r="AC41" t="str">
@@ -37002,7 +37050,7 @@
         <v>tc-2.00.df-N.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="H42" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC42,AB42:AB42)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y42:AA42)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-N.dm-Lo.cp-00.CF1</v>
       </c>
       <c r="I42" t="str">
@@ -37021,9 +37069,9 @@
         <f t="shared" si="21"/>
         <v>N</v>
       </c>
-      <c r="M42">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M42" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O42">
         <v>5</v>
@@ -37053,7 +37101,7 @@
         <v>2</v>
       </c>
       <c r="Y42" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Lo</v>
       </c>
       <c r="Z42" t="str">
@@ -37061,11 +37109,11 @@
         <v>cp-00</v>
       </c>
       <c r="AA42" t="str">
+        <f t="shared" si="23"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB42" t="str">
         <f t="shared" si="24"/>
-        <v>CF1</v>
-      </c>
-      <c r="AB42" t="str">
-        <f t="shared" si="25"/>
         <v>df-N</v>
       </c>
       <c r="AC42" t="str">
@@ -37083,7 +37131,7 @@
         <v>tc-2.00.df-N.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="H43" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC43,AB43:AB43)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y43:AA43)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-N.dm-Hi.cp-00.CF1</v>
       </c>
       <c r="I43" t="str">
@@ -37102,9 +37150,9 @@
         <f t="shared" si="21"/>
         <v>N</v>
       </c>
-      <c r="M43">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M43" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O43">
         <v>5</v>
@@ -37134,7 +37182,7 @@
         <v>2</v>
       </c>
       <c r="Y43" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Hi</v>
       </c>
       <c r="Z43" t="str">
@@ -37142,11 +37190,11 @@
         <v>cp-00</v>
       </c>
       <c r="AA43" t="str">
+        <f t="shared" si="23"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB43" t="str">
         <f t="shared" si="24"/>
-        <v>CF1</v>
-      </c>
-      <c r="AB43" t="str">
-        <f t="shared" si="25"/>
         <v>df-N</v>
       </c>
       <c r="AC43" t="str">
@@ -37164,7 +37212,7 @@
         <v>tc-2.00.df-N.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="H44" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC44,AB44:AB44)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y44:AA44)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-N.dm-Lo.cp-95.CF1</v>
       </c>
       <c r="I44" t="str">
@@ -37183,9 +37231,9 @@
         <f t="shared" si="21"/>
         <v>N</v>
       </c>
-      <c r="M44">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M44" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O44">
         <v>5</v>
@@ -37215,7 +37263,7 @@
         <v>2</v>
       </c>
       <c r="Y44" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Lo</v>
       </c>
       <c r="Z44" t="str">
@@ -37223,11 +37271,11 @@
         <v>cp-95</v>
       </c>
       <c r="AA44" t="str">
+        <f t="shared" si="23"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB44" t="str">
         <f t="shared" si="24"/>
-        <v>CF1</v>
-      </c>
-      <c r="AB44" t="str">
-        <f t="shared" si="25"/>
         <v>df-N</v>
       </c>
       <c r="AC44" t="str">
@@ -37245,7 +37293,7 @@
         <v>tc-2.00.df-N.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="H45" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC45,AB45:AB45)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y45:AA45)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-N.dm-Hi.cp-95.CF1</v>
       </c>
       <c r="I45" t="str">
@@ -37264,9 +37312,9 @@
         <f t="shared" si="21"/>
         <v>N</v>
       </c>
-      <c r="M45">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M45" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O45">
         <v>5</v>
@@ -37296,7 +37344,7 @@
         <v>2</v>
       </c>
       <c r="Y45" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Hi</v>
       </c>
       <c r="Z45" t="str">
@@ -37304,11 +37352,11 @@
         <v>cp-95</v>
       </c>
       <c r="AA45" t="str">
+        <f t="shared" si="23"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB45" t="str">
         <f t="shared" si="24"/>
-        <v>CF1</v>
-      </c>
-      <c r="AB45" t="str">
-        <f t="shared" si="25"/>
         <v>df-N</v>
       </c>
       <c r="AC45" t="str">
@@ -37326,7 +37374,7 @@
         <v>tc-2.00.df-Y.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="H46" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC46,AB46:AB46)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y46:AA46)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-Y.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="I46" t="str">
@@ -37345,9 +37393,9 @@
         <f t="shared" si="21"/>
         <v>Y</v>
       </c>
-      <c r="M46">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M46" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O46">
         <v>5</v>
@@ -37377,7 +37425,7 @@
         <v>2</v>
       </c>
       <c r="Y46" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Lo</v>
       </c>
       <c r="Z46" t="str">
@@ -37385,11 +37433,11 @@
         <v>cp-00</v>
       </c>
       <c r="AA46" t="str">
+        <f t="shared" si="23"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB46" t="str">
         <f t="shared" si="24"/>
-        <v>CF6</v>
-      </c>
-      <c r="AB46" t="str">
-        <f t="shared" si="25"/>
         <v>df-Y</v>
       </c>
       <c r="AC46" t="str">
@@ -37407,7 +37455,7 @@
         <v>tc-2.00.df-Y.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="H47" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC47,AB47:AB47)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y47:AA47)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-Y.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="I47" t="str">
@@ -37426,9 +37474,9 @@
         <f t="shared" si="21"/>
         <v>Y</v>
       </c>
-      <c r="M47">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M47" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O47">
         <v>5</v>
@@ -37458,7 +37506,7 @@
         <v>2</v>
       </c>
       <c r="Y47" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Hi</v>
       </c>
       <c r="Z47" t="str">
@@ -37466,11 +37514,11 @@
         <v>cp-00</v>
       </c>
       <c r="AA47" t="str">
+        <f t="shared" si="23"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB47" t="str">
         <f t="shared" si="24"/>
-        <v>CF6</v>
-      </c>
-      <c r="AB47" t="str">
-        <f t="shared" si="25"/>
         <v>df-Y</v>
       </c>
       <c r="AC47" t="str">
@@ -37488,7 +37536,7 @@
         <v>tc-2.00.df-Y.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="H48" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC48,AB48:AB48)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y48:AA48)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-Y.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="I48" t="str">
@@ -37507,9 +37555,9 @@
         <f t="shared" si="21"/>
         <v>Y</v>
       </c>
-      <c r="M48">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M48" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O48">
         <v>5</v>
@@ -37539,7 +37587,7 @@
         <v>2</v>
       </c>
       <c r="Y48" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Lo</v>
       </c>
       <c r="Z48" t="str">
@@ -37547,11 +37595,11 @@
         <v>cp-95</v>
       </c>
       <c r="AA48" t="str">
+        <f t="shared" si="23"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB48" t="str">
         <f t="shared" si="24"/>
-        <v>CF6</v>
-      </c>
-      <c r="AB48" t="str">
-        <f t="shared" si="25"/>
         <v>df-Y</v>
       </c>
       <c r="AC48" t="str">
@@ -37569,7 +37617,7 @@
         <v>tc-2.00.df-Y.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="H49" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC49,AB49:AB49)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y49:AA49)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-Y.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="I49" t="str">
@@ -37588,9 +37636,9 @@
         <f t="shared" si="21"/>
         <v>Y</v>
       </c>
-      <c r="M49">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M49" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O49">
         <v>5</v>
@@ -37620,7 +37668,7 @@
         <v>2</v>
       </c>
       <c r="Y49" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Hi</v>
       </c>
       <c r="Z49" t="str">
@@ -37628,11 +37676,11 @@
         <v>cp-95</v>
       </c>
       <c r="AA49" t="str">
+        <f t="shared" si="23"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB49" t="str">
         <f t="shared" si="24"/>
-        <v>CF6</v>
-      </c>
-      <c r="AB49" t="str">
-        <f t="shared" si="25"/>
         <v>df-Y</v>
       </c>
       <c r="AC49" t="str">
@@ -37650,7 +37698,7 @@
         <v>tc-2.00.df-N.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="H50" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC50,AB50:AB50)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y50:AA50)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-N.dm-Lo.cp-00.CF6</v>
       </c>
       <c r="I50" t="str">
@@ -37669,9 +37717,9 @@
         <f t="shared" si="21"/>
         <v>N</v>
       </c>
-      <c r="M50">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M50" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O50">
         <v>5</v>
@@ -37701,7 +37749,7 @@
         <v>2</v>
       </c>
       <c r="Y50" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Lo</v>
       </c>
       <c r="Z50" t="str">
@@ -37709,11 +37757,11 @@
         <v>cp-00</v>
       </c>
       <c r="AA50" t="str">
+        <f t="shared" si="23"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB50" t="str">
         <f t="shared" si="24"/>
-        <v>CF6</v>
-      </c>
-      <c r="AB50" t="str">
-        <f t="shared" si="25"/>
         <v>df-N</v>
       </c>
       <c r="AC50" t="str">
@@ -37731,7 +37779,7 @@
         <v>tc-2.00.df-N.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="H51" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC51,AB51:AB51)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y51:AA51)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-N.dm-Hi.cp-00.CF6</v>
       </c>
       <c r="I51" t="str">
@@ -37750,9 +37798,9 @@
         <f t="shared" si="21"/>
         <v>N</v>
       </c>
-      <c r="M51">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M51" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O51">
         <v>5</v>
@@ -37782,7 +37830,7 @@
         <v>2</v>
       </c>
       <c r="Y51" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Hi</v>
       </c>
       <c r="Z51" t="str">
@@ -37790,11 +37838,11 @@
         <v>cp-00</v>
       </c>
       <c r="AA51" t="str">
+        <f t="shared" si="23"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB51" t="str">
         <f t="shared" si="24"/>
-        <v>CF6</v>
-      </c>
-      <c r="AB51" t="str">
-        <f t="shared" si="25"/>
         <v>df-N</v>
       </c>
       <c r="AC51" t="str">
@@ -37812,7 +37860,7 @@
         <v>tc-2.00.df-N.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="H52" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC52,AB52:AB52)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y52:AA52)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-N.dm-Lo.cp-95.CF6</v>
       </c>
       <c r="I52" t="str">
@@ -37831,9 +37879,9 @@
         <f t="shared" si="21"/>
         <v>N</v>
       </c>
-      <c r="M52">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M52" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O52">
         <v>5</v>
@@ -37863,7 +37911,7 @@
         <v>2</v>
       </c>
       <c r="Y52" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Lo</v>
       </c>
       <c r="Z52" t="str">
@@ -37871,11 +37919,11 @@
         <v>cp-95</v>
       </c>
       <c r="AA52" t="str">
+        <f t="shared" si="23"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB52" t="str">
         <f t="shared" si="24"/>
-        <v>CF6</v>
-      </c>
-      <c r="AB52" t="str">
-        <f t="shared" si="25"/>
         <v>df-N</v>
       </c>
       <c r="AC52" t="str">
@@ -37893,7 +37941,7 @@
         <v>tc-2.00.df-N.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="H53" t="str">
-        <f>_xlfn.TEXTJOIN(".",TRUE,AC53,AB53:AB53)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y53:AA53)</f>
+        <f t="shared" si="1"/>
         <v>tc-2.00.df-N.dm-Hi.cp-95.CF6</v>
       </c>
       <c r="I53" t="str">
@@ -37912,9 +37960,9 @@
         <f t="shared" si="21"/>
         <v>N</v>
       </c>
-      <c r="M53">
-        <f t="shared" si="22"/>
-        <v>2</v>
+      <c r="M53" t="str">
+        <f t="shared" si="8"/>
+        <v>2.00</v>
       </c>
       <c r="O53">
         <v>5</v>
@@ -37944,7 +37992,7 @@
         <v>2</v>
       </c>
       <c r="Y53" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="22"/>
         <v>dm-Hi</v>
       </c>
       <c r="Z53" t="str">
@@ -37952,16 +38000,1312 @@
         <v>cp-95</v>
       </c>
       <c r="AA53" t="str">
+        <f t="shared" si="23"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB53" t="str">
         <f t="shared" si="24"/>
-        <v>CF6</v>
-      </c>
-      <c r="AB53" t="str">
-        <f t="shared" si="25"/>
         <v>df-N</v>
       </c>
       <c r="AC53" t="str">
         <f t="shared" si="13"/>
         <v>tc-2.00</v>
+      </c>
+    </row>
+    <row r="54" spans="2:29">
+      <c r="B54" t="str">
+        <f t="shared" ref="B54:B69" si="25">"vs~"&amp;TEXT(Q54,"0000")</f>
+        <v>vs~0049</v>
+      </c>
+      <c r="C54" t="str">
+        <f t="shared" ref="C54:C69" si="26">H54</f>
+        <v>tc-0.10.df-Y.dm-Lo.cp-00.CF1</v>
+      </c>
+      <c r="H54" t="str">
+        <f t="shared" ref="H54:H69" si="27">_xlfn.TEXTJOIN(".",TRUE,AC54,AB54:AB54)&amp;"."&amp;_xlfn.TEXTJOIN(".",TRUE,Y54:AA54)</f>
+        <v>tc-0.10.df-Y.dm-Lo.cp-00.CF1</v>
+      </c>
+      <c r="I54" t="str">
+        <f t="shared" ref="I54:I69" si="28">R54</f>
+        <v>Lo</v>
+      </c>
+      <c r="J54" t="str">
+        <f t="shared" ref="J54:J69" si="29">TEXT(S54,"00")</f>
+        <v>00</v>
+      </c>
+      <c r="K54" t="str">
+        <f t="shared" ref="K54:K69" si="30">T54</f>
+        <v>CF1</v>
+      </c>
+      <c r="L54" t="str">
+        <f t="shared" ref="L54:L69" si="31">U54</f>
+        <v>Y</v>
+      </c>
+      <c r="M54" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O54">
+        <v>5</v>
+      </c>
+      <c r="P54" t="s">
+        <v>1156</v>
+      </c>
+      <c r="Q54">
+        <v>49</v>
+      </c>
+      <c r="R54" t="s">
+        <v>1092</v>
+      </c>
+      <c r="S54">
+        <v>0</v>
+      </c>
+      <c r="T54" t="s">
+        <v>1087</v>
+      </c>
+      <c r="U54" t="s">
+        <v>1093</v>
+      </c>
+      <c r="V54" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W54">
+        <v>0.1</v>
+      </c>
+      <c r="Y54" t="str">
+        <f t="shared" ref="Y54:Y69" si="32">R$1&amp;"-"&amp;R54</f>
+        <v>dm-Lo</v>
+      </c>
+      <c r="Z54" t="str">
+        <f t="shared" ref="Z54:Z69" si="33">S$1&amp;"-"&amp;TEXT(S54,"00")</f>
+        <v>cp-00</v>
+      </c>
+      <c r="AA54" t="str">
+        <f t="shared" ref="AA54:AA69" si="34">T54</f>
+        <v>CF1</v>
+      </c>
+      <c r="AB54" t="str">
+        <f t="shared" ref="AB54:AB69" si="35">U$1&amp;"-"&amp;U54</f>
+        <v>df-Y</v>
+      </c>
+      <c r="AC54" t="str">
+        <f t="shared" ref="AC54:AC69" si="36">W$1&amp;"-"&amp;TEXT(W54,"0.00")</f>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="55" spans="2:29">
+      <c r="B55" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0050</v>
+      </c>
+      <c r="C55" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-Y.dm-Hi.cp-00.CF1</v>
+      </c>
+      <c r="H55" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-Y.dm-Hi.cp-00.CF1</v>
+      </c>
+      <c r="I55" t="str">
+        <f t="shared" si="28"/>
+        <v>Hi</v>
+      </c>
+      <c r="J55" t="str">
+        <f t="shared" si="29"/>
+        <v>00</v>
+      </c>
+      <c r="K55" t="str">
+        <f t="shared" si="30"/>
+        <v>CF1</v>
+      </c>
+      <c r="L55" t="str">
+        <f t="shared" si="31"/>
+        <v>Y</v>
+      </c>
+      <c r="M55" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O55">
+        <v>5</v>
+      </c>
+      <c r="P55" t="s">
+        <v>1157</v>
+      </c>
+      <c r="Q55">
+        <v>50</v>
+      </c>
+      <c r="R55" t="s">
+        <v>1094</v>
+      </c>
+      <c r="S55">
+        <v>0</v>
+      </c>
+      <c r="T55" t="s">
+        <v>1087</v>
+      </c>
+      <c r="U55" t="s">
+        <v>1093</v>
+      </c>
+      <c r="V55" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W55">
+        <v>0.1</v>
+      </c>
+      <c r="Y55" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Hi</v>
+      </c>
+      <c r="Z55" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-00</v>
+      </c>
+      <c r="AA55" t="str">
+        <f t="shared" si="34"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB55" t="str">
+        <f t="shared" si="35"/>
+        <v>df-Y</v>
+      </c>
+      <c r="AC55" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="56" spans="2:29">
+      <c r="B56" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0051</v>
+      </c>
+      <c r="C56" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-Y.dm-Lo.cp-95.CF1</v>
+      </c>
+      <c r="H56" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-Y.dm-Lo.cp-95.CF1</v>
+      </c>
+      <c r="I56" t="str">
+        <f t="shared" si="28"/>
+        <v>Lo</v>
+      </c>
+      <c r="J56" t="str">
+        <f t="shared" si="29"/>
+        <v>95</v>
+      </c>
+      <c r="K56" t="str">
+        <f t="shared" si="30"/>
+        <v>CF1</v>
+      </c>
+      <c r="L56" t="str">
+        <f t="shared" si="31"/>
+        <v>Y</v>
+      </c>
+      <c r="M56" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O56">
+        <v>5</v>
+      </c>
+      <c r="P56" t="s">
+        <v>1158</v>
+      </c>
+      <c r="Q56">
+        <v>51</v>
+      </c>
+      <c r="R56" t="s">
+        <v>1092</v>
+      </c>
+      <c r="S56">
+        <v>95</v>
+      </c>
+      <c r="T56" t="s">
+        <v>1087</v>
+      </c>
+      <c r="U56" t="s">
+        <v>1093</v>
+      </c>
+      <c r="V56" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W56">
+        <v>0.1</v>
+      </c>
+      <c r="Y56" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Lo</v>
+      </c>
+      <c r="Z56" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-95</v>
+      </c>
+      <c r="AA56" t="str">
+        <f t="shared" si="34"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB56" t="str">
+        <f t="shared" si="35"/>
+        <v>df-Y</v>
+      </c>
+      <c r="AC56" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="57" spans="2:29">
+      <c r="B57" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0052</v>
+      </c>
+      <c r="C57" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-Y.dm-Hi.cp-95.CF1</v>
+      </c>
+      <c r="H57" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-Y.dm-Hi.cp-95.CF1</v>
+      </c>
+      <c r="I57" t="str">
+        <f t="shared" si="28"/>
+        <v>Hi</v>
+      </c>
+      <c r="J57" t="str">
+        <f t="shared" si="29"/>
+        <v>95</v>
+      </c>
+      <c r="K57" t="str">
+        <f t="shared" si="30"/>
+        <v>CF1</v>
+      </c>
+      <c r="L57" t="str">
+        <f t="shared" si="31"/>
+        <v>Y</v>
+      </c>
+      <c r="M57" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O57">
+        <v>5</v>
+      </c>
+      <c r="P57" t="s">
+        <v>1159</v>
+      </c>
+      <c r="Q57">
+        <v>52</v>
+      </c>
+      <c r="R57" t="s">
+        <v>1094</v>
+      </c>
+      <c r="S57">
+        <v>95</v>
+      </c>
+      <c r="T57" t="s">
+        <v>1087</v>
+      </c>
+      <c r="U57" t="s">
+        <v>1093</v>
+      </c>
+      <c r="V57" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W57">
+        <v>0.1</v>
+      </c>
+      <c r="Y57" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Hi</v>
+      </c>
+      <c r="Z57" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-95</v>
+      </c>
+      <c r="AA57" t="str">
+        <f t="shared" si="34"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB57" t="str">
+        <f t="shared" si="35"/>
+        <v>df-Y</v>
+      </c>
+      <c r="AC57" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="58" spans="2:29">
+      <c r="B58" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0053</v>
+      </c>
+      <c r="C58" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-N.dm-Lo.cp-00.CF1</v>
+      </c>
+      <c r="H58" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-N.dm-Lo.cp-00.CF1</v>
+      </c>
+      <c r="I58" t="str">
+        <f t="shared" si="28"/>
+        <v>Lo</v>
+      </c>
+      <c r="J58" t="str">
+        <f t="shared" si="29"/>
+        <v>00</v>
+      </c>
+      <c r="K58" t="str">
+        <f t="shared" si="30"/>
+        <v>CF1</v>
+      </c>
+      <c r="L58" t="str">
+        <f t="shared" si="31"/>
+        <v>N</v>
+      </c>
+      <c r="M58" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O58">
+        <v>5</v>
+      </c>
+      <c r="P58" t="s">
+        <v>1160</v>
+      </c>
+      <c r="Q58">
+        <v>53</v>
+      </c>
+      <c r="R58" t="s">
+        <v>1092</v>
+      </c>
+      <c r="S58">
+        <v>0</v>
+      </c>
+      <c r="T58" t="s">
+        <v>1087</v>
+      </c>
+      <c r="U58" t="s">
+        <v>1095</v>
+      </c>
+      <c r="V58" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W58">
+        <v>0.1</v>
+      </c>
+      <c r="Y58" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Lo</v>
+      </c>
+      <c r="Z58" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-00</v>
+      </c>
+      <c r="AA58" t="str">
+        <f t="shared" si="34"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB58" t="str">
+        <f t="shared" si="35"/>
+        <v>df-N</v>
+      </c>
+      <c r="AC58" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="59" spans="2:29">
+      <c r="B59" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0054</v>
+      </c>
+      <c r="C59" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-N.dm-Hi.cp-00.CF1</v>
+      </c>
+      <c r="H59" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-N.dm-Hi.cp-00.CF1</v>
+      </c>
+      <c r="I59" t="str">
+        <f t="shared" si="28"/>
+        <v>Hi</v>
+      </c>
+      <c r="J59" t="str">
+        <f t="shared" si="29"/>
+        <v>00</v>
+      </c>
+      <c r="K59" t="str">
+        <f t="shared" si="30"/>
+        <v>CF1</v>
+      </c>
+      <c r="L59" t="str">
+        <f t="shared" si="31"/>
+        <v>N</v>
+      </c>
+      <c r="M59" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O59">
+        <v>5</v>
+      </c>
+      <c r="P59" t="s">
+        <v>1161</v>
+      </c>
+      <c r="Q59">
+        <v>54</v>
+      </c>
+      <c r="R59" t="s">
+        <v>1094</v>
+      </c>
+      <c r="S59">
+        <v>0</v>
+      </c>
+      <c r="T59" t="s">
+        <v>1087</v>
+      </c>
+      <c r="U59" t="s">
+        <v>1095</v>
+      </c>
+      <c r="V59" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W59">
+        <v>0.1</v>
+      </c>
+      <c r="Y59" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Hi</v>
+      </c>
+      <c r="Z59" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-00</v>
+      </c>
+      <c r="AA59" t="str">
+        <f t="shared" si="34"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB59" t="str">
+        <f t="shared" si="35"/>
+        <v>df-N</v>
+      </c>
+      <c r="AC59" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="60" spans="2:29">
+      <c r="B60" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0055</v>
+      </c>
+      <c r="C60" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-N.dm-Lo.cp-95.CF1</v>
+      </c>
+      <c r="H60" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-N.dm-Lo.cp-95.CF1</v>
+      </c>
+      <c r="I60" t="str">
+        <f t="shared" si="28"/>
+        <v>Lo</v>
+      </c>
+      <c r="J60" t="str">
+        <f t="shared" si="29"/>
+        <v>95</v>
+      </c>
+      <c r="K60" t="str">
+        <f t="shared" si="30"/>
+        <v>CF1</v>
+      </c>
+      <c r="L60" t="str">
+        <f t="shared" si="31"/>
+        <v>N</v>
+      </c>
+      <c r="M60" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O60">
+        <v>5</v>
+      </c>
+      <c r="P60" t="s">
+        <v>1162</v>
+      </c>
+      <c r="Q60">
+        <v>55</v>
+      </c>
+      <c r="R60" t="s">
+        <v>1092</v>
+      </c>
+      <c r="S60">
+        <v>95</v>
+      </c>
+      <c r="T60" t="s">
+        <v>1087</v>
+      </c>
+      <c r="U60" t="s">
+        <v>1095</v>
+      </c>
+      <c r="V60" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W60">
+        <v>0.1</v>
+      </c>
+      <c r="Y60" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Lo</v>
+      </c>
+      <c r="Z60" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-95</v>
+      </c>
+      <c r="AA60" t="str">
+        <f t="shared" si="34"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB60" t="str">
+        <f t="shared" si="35"/>
+        <v>df-N</v>
+      </c>
+      <c r="AC60" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="61" spans="2:29">
+      <c r="B61" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0056</v>
+      </c>
+      <c r="C61" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-N.dm-Hi.cp-95.CF1</v>
+      </c>
+      <c r="H61" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-N.dm-Hi.cp-95.CF1</v>
+      </c>
+      <c r="I61" t="str">
+        <f t="shared" si="28"/>
+        <v>Hi</v>
+      </c>
+      <c r="J61" t="str">
+        <f t="shared" si="29"/>
+        <v>95</v>
+      </c>
+      <c r="K61" t="str">
+        <f t="shared" si="30"/>
+        <v>CF1</v>
+      </c>
+      <c r="L61" t="str">
+        <f t="shared" si="31"/>
+        <v>N</v>
+      </c>
+      <c r="M61" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O61">
+        <v>5</v>
+      </c>
+      <c r="P61" t="s">
+        <v>1163</v>
+      </c>
+      <c r="Q61">
+        <v>56</v>
+      </c>
+      <c r="R61" t="s">
+        <v>1094</v>
+      </c>
+      <c r="S61">
+        <v>95</v>
+      </c>
+      <c r="T61" t="s">
+        <v>1087</v>
+      </c>
+      <c r="U61" t="s">
+        <v>1095</v>
+      </c>
+      <c r="V61" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W61">
+        <v>0.1</v>
+      </c>
+      <c r="Y61" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Hi</v>
+      </c>
+      <c r="Z61" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-95</v>
+      </c>
+      <c r="AA61" t="str">
+        <f t="shared" si="34"/>
+        <v>CF1</v>
+      </c>
+      <c r="AB61" t="str">
+        <f t="shared" si="35"/>
+        <v>df-N</v>
+      </c>
+      <c r="AC61" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="62" spans="2:29">
+      <c r="B62" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0057</v>
+      </c>
+      <c r="C62" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-Y.dm-Lo.cp-00.CF6</v>
+      </c>
+      <c r="H62" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-Y.dm-Lo.cp-00.CF6</v>
+      </c>
+      <c r="I62" t="str">
+        <f t="shared" si="28"/>
+        <v>Lo</v>
+      </c>
+      <c r="J62" t="str">
+        <f t="shared" si="29"/>
+        <v>00</v>
+      </c>
+      <c r="K62" t="str">
+        <f t="shared" si="30"/>
+        <v>CF6</v>
+      </c>
+      <c r="L62" t="str">
+        <f t="shared" si="31"/>
+        <v>Y</v>
+      </c>
+      <c r="M62" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O62">
+        <v>5</v>
+      </c>
+      <c r="P62" t="s">
+        <v>1164</v>
+      </c>
+      <c r="Q62">
+        <v>57</v>
+      </c>
+      <c r="R62" t="s">
+        <v>1092</v>
+      </c>
+      <c r="S62">
+        <v>0</v>
+      </c>
+      <c r="T62" t="s">
+        <v>1088</v>
+      </c>
+      <c r="U62" t="s">
+        <v>1093</v>
+      </c>
+      <c r="V62" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W62">
+        <v>0.1</v>
+      </c>
+      <c r="Y62" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Lo</v>
+      </c>
+      <c r="Z62" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-00</v>
+      </c>
+      <c r="AA62" t="str">
+        <f t="shared" si="34"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB62" t="str">
+        <f t="shared" si="35"/>
+        <v>df-Y</v>
+      </c>
+      <c r="AC62" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="63" spans="2:29">
+      <c r="B63" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0058</v>
+      </c>
+      <c r="C63" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-Y.dm-Hi.cp-00.CF6</v>
+      </c>
+      <c r="H63" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-Y.dm-Hi.cp-00.CF6</v>
+      </c>
+      <c r="I63" t="str">
+        <f t="shared" si="28"/>
+        <v>Hi</v>
+      </c>
+      <c r="J63" t="str">
+        <f t="shared" si="29"/>
+        <v>00</v>
+      </c>
+      <c r="K63" t="str">
+        <f t="shared" si="30"/>
+        <v>CF6</v>
+      </c>
+      <c r="L63" t="str">
+        <f t="shared" si="31"/>
+        <v>Y</v>
+      </c>
+      <c r="M63" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O63">
+        <v>5</v>
+      </c>
+      <c r="P63" t="s">
+        <v>1165</v>
+      </c>
+      <c r="Q63">
+        <v>58</v>
+      </c>
+      <c r="R63" t="s">
+        <v>1094</v>
+      </c>
+      <c r="S63">
+        <v>0</v>
+      </c>
+      <c r="T63" t="s">
+        <v>1088</v>
+      </c>
+      <c r="U63" t="s">
+        <v>1093</v>
+      </c>
+      <c r="V63" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W63">
+        <v>0.1</v>
+      </c>
+      <c r="Y63" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Hi</v>
+      </c>
+      <c r="Z63" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-00</v>
+      </c>
+      <c r="AA63" t="str">
+        <f t="shared" si="34"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB63" t="str">
+        <f t="shared" si="35"/>
+        <v>df-Y</v>
+      </c>
+      <c r="AC63" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="64" spans="2:29">
+      <c r="B64" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0059</v>
+      </c>
+      <c r="C64" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-Y.dm-Lo.cp-95.CF6</v>
+      </c>
+      <c r="H64" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-Y.dm-Lo.cp-95.CF6</v>
+      </c>
+      <c r="I64" t="str">
+        <f t="shared" si="28"/>
+        <v>Lo</v>
+      </c>
+      <c r="J64" t="str">
+        <f t="shared" si="29"/>
+        <v>95</v>
+      </c>
+      <c r="K64" t="str">
+        <f t="shared" si="30"/>
+        <v>CF6</v>
+      </c>
+      <c r="L64" t="str">
+        <f t="shared" si="31"/>
+        <v>Y</v>
+      </c>
+      <c r="M64" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O64">
+        <v>5</v>
+      </c>
+      <c r="P64" t="s">
+        <v>1166</v>
+      </c>
+      <c r="Q64">
+        <v>59</v>
+      </c>
+      <c r="R64" t="s">
+        <v>1092</v>
+      </c>
+      <c r="S64">
+        <v>95</v>
+      </c>
+      <c r="T64" t="s">
+        <v>1088</v>
+      </c>
+      <c r="U64" t="s">
+        <v>1093</v>
+      </c>
+      <c r="V64" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W64">
+        <v>0.1</v>
+      </c>
+      <c r="Y64" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Lo</v>
+      </c>
+      <c r="Z64" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-95</v>
+      </c>
+      <c r="AA64" t="str">
+        <f t="shared" si="34"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB64" t="str">
+        <f t="shared" si="35"/>
+        <v>df-Y</v>
+      </c>
+      <c r="AC64" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="65" spans="2:29">
+      <c r="B65" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0060</v>
+      </c>
+      <c r="C65" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-Y.dm-Hi.cp-95.CF6</v>
+      </c>
+      <c r="H65" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-Y.dm-Hi.cp-95.CF6</v>
+      </c>
+      <c r="I65" t="str">
+        <f t="shared" si="28"/>
+        <v>Hi</v>
+      </c>
+      <c r="J65" t="str">
+        <f t="shared" si="29"/>
+        <v>95</v>
+      </c>
+      <c r="K65" t="str">
+        <f t="shared" si="30"/>
+        <v>CF6</v>
+      </c>
+      <c r="L65" t="str">
+        <f t="shared" si="31"/>
+        <v>Y</v>
+      </c>
+      <c r="M65" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O65">
+        <v>5</v>
+      </c>
+      <c r="P65" t="s">
+        <v>1167</v>
+      </c>
+      <c r="Q65">
+        <v>60</v>
+      </c>
+      <c r="R65" t="s">
+        <v>1094</v>
+      </c>
+      <c r="S65">
+        <v>95</v>
+      </c>
+      <c r="T65" t="s">
+        <v>1088</v>
+      </c>
+      <c r="U65" t="s">
+        <v>1093</v>
+      </c>
+      <c r="V65" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W65">
+        <v>0.1</v>
+      </c>
+      <c r="Y65" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Hi</v>
+      </c>
+      <c r="Z65" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-95</v>
+      </c>
+      <c r="AA65" t="str">
+        <f t="shared" si="34"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB65" t="str">
+        <f t="shared" si="35"/>
+        <v>df-Y</v>
+      </c>
+      <c r="AC65" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="66" spans="2:29">
+      <c r="B66" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0061</v>
+      </c>
+      <c r="C66" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-N.dm-Lo.cp-00.CF6</v>
+      </c>
+      <c r="H66" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-N.dm-Lo.cp-00.CF6</v>
+      </c>
+      <c r="I66" t="str">
+        <f t="shared" si="28"/>
+        <v>Lo</v>
+      </c>
+      <c r="J66" t="str">
+        <f t="shared" si="29"/>
+        <v>00</v>
+      </c>
+      <c r="K66" t="str">
+        <f t="shared" si="30"/>
+        <v>CF6</v>
+      </c>
+      <c r="L66" t="str">
+        <f t="shared" si="31"/>
+        <v>N</v>
+      </c>
+      <c r="M66" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O66">
+        <v>5</v>
+      </c>
+      <c r="P66" t="s">
+        <v>1168</v>
+      </c>
+      <c r="Q66">
+        <v>61</v>
+      </c>
+      <c r="R66" t="s">
+        <v>1092</v>
+      </c>
+      <c r="S66">
+        <v>0</v>
+      </c>
+      <c r="T66" t="s">
+        <v>1088</v>
+      </c>
+      <c r="U66" t="s">
+        <v>1095</v>
+      </c>
+      <c r="V66" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W66">
+        <v>0.1</v>
+      </c>
+      <c r="Y66" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Lo</v>
+      </c>
+      <c r="Z66" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-00</v>
+      </c>
+      <c r="AA66" t="str">
+        <f t="shared" si="34"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB66" t="str">
+        <f t="shared" si="35"/>
+        <v>df-N</v>
+      </c>
+      <c r="AC66" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="67" spans="2:29">
+      <c r="B67" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0062</v>
+      </c>
+      <c r="C67" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-N.dm-Hi.cp-00.CF6</v>
+      </c>
+      <c r="H67" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-N.dm-Hi.cp-00.CF6</v>
+      </c>
+      <c r="I67" t="str">
+        <f t="shared" si="28"/>
+        <v>Hi</v>
+      </c>
+      <c r="J67" t="str">
+        <f t="shared" si="29"/>
+        <v>00</v>
+      </c>
+      <c r="K67" t="str">
+        <f t="shared" si="30"/>
+        <v>CF6</v>
+      </c>
+      <c r="L67" t="str">
+        <f t="shared" si="31"/>
+        <v>N</v>
+      </c>
+      <c r="M67" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O67">
+        <v>5</v>
+      </c>
+      <c r="P67" t="s">
+        <v>1169</v>
+      </c>
+      <c r="Q67">
+        <v>62</v>
+      </c>
+      <c r="R67" t="s">
+        <v>1094</v>
+      </c>
+      <c r="S67">
+        <v>0</v>
+      </c>
+      <c r="T67" t="s">
+        <v>1088</v>
+      </c>
+      <c r="U67" t="s">
+        <v>1095</v>
+      </c>
+      <c r="V67" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W67">
+        <v>0.1</v>
+      </c>
+      <c r="Y67" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Hi</v>
+      </c>
+      <c r="Z67" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-00</v>
+      </c>
+      <c r="AA67" t="str">
+        <f t="shared" si="34"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB67" t="str">
+        <f t="shared" si="35"/>
+        <v>df-N</v>
+      </c>
+      <c r="AC67" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="68" spans="2:29">
+      <c r="B68" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0063</v>
+      </c>
+      <c r="C68" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-N.dm-Lo.cp-95.CF6</v>
+      </c>
+      <c r="H68" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-N.dm-Lo.cp-95.CF6</v>
+      </c>
+      <c r="I68" t="str">
+        <f t="shared" si="28"/>
+        <v>Lo</v>
+      </c>
+      <c r="J68" t="str">
+        <f t="shared" si="29"/>
+        <v>95</v>
+      </c>
+      <c r="K68" t="str">
+        <f t="shared" si="30"/>
+        <v>CF6</v>
+      </c>
+      <c r="L68" t="str">
+        <f t="shared" si="31"/>
+        <v>N</v>
+      </c>
+      <c r="M68" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O68">
+        <v>5</v>
+      </c>
+      <c r="P68" t="s">
+        <v>1170</v>
+      </c>
+      <c r="Q68">
+        <v>63</v>
+      </c>
+      <c r="R68" t="s">
+        <v>1092</v>
+      </c>
+      <c r="S68">
+        <v>95</v>
+      </c>
+      <c r="T68" t="s">
+        <v>1088</v>
+      </c>
+      <c r="U68" t="s">
+        <v>1095</v>
+      </c>
+      <c r="V68" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W68">
+        <v>0.1</v>
+      </c>
+      <c r="Y68" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Lo</v>
+      </c>
+      <c r="Z68" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-95</v>
+      </c>
+      <c r="AA68" t="str">
+        <f t="shared" si="34"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB68" t="str">
+        <f t="shared" si="35"/>
+        <v>df-N</v>
+      </c>
+      <c r="AC68" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
+      </c>
+    </row>
+    <row r="69" spans="2:29">
+      <c r="B69" t="str">
+        <f t="shared" si="25"/>
+        <v>vs~0064</v>
+      </c>
+      <c r="C69" t="str">
+        <f t="shared" si="26"/>
+        <v>tc-0.10.df-N.dm-Hi.cp-95.CF6</v>
+      </c>
+      <c r="H69" t="str">
+        <f t="shared" si="27"/>
+        <v>tc-0.10.df-N.dm-Hi.cp-95.CF6</v>
+      </c>
+      <c r="I69" t="str">
+        <f t="shared" si="28"/>
+        <v>Hi</v>
+      </c>
+      <c r="J69" t="str">
+        <f t="shared" si="29"/>
+        <v>95</v>
+      </c>
+      <c r="K69" t="str">
+        <f t="shared" si="30"/>
+        <v>CF6</v>
+      </c>
+      <c r="L69" t="str">
+        <f t="shared" si="31"/>
+        <v>N</v>
+      </c>
+      <c r="M69" t="str">
+        <f t="shared" si="8"/>
+        <v>0.10</v>
+      </c>
+      <c r="O69">
+        <v>5</v>
+      </c>
+      <c r="P69" t="s">
+        <v>1171</v>
+      </c>
+      <c r="Q69">
+        <v>64</v>
+      </c>
+      <c r="R69" t="s">
+        <v>1094</v>
+      </c>
+      <c r="S69">
+        <v>95</v>
+      </c>
+      <c r="T69" t="s">
+        <v>1088</v>
+      </c>
+      <c r="U69" t="s">
+        <v>1095</v>
+      </c>
+      <c r="V69" t="s">
+        <v>1093</v>
+      </c>
+      <c r="W69">
+        <v>0.1</v>
+      </c>
+      <c r="Y69" t="str">
+        <f t="shared" si="32"/>
+        <v>dm-Hi</v>
+      </c>
+      <c r="Z69" t="str">
+        <f t="shared" si="33"/>
+        <v>cp-95</v>
+      </c>
+      <c r="AA69" t="str">
+        <f t="shared" si="34"/>
+        <v>CF6</v>
+      </c>
+      <c r="AB69" t="str">
+        <f t="shared" si="35"/>
+        <v>df-N</v>
+      </c>
+      <c r="AC69" t="str">
+        <f t="shared" si="36"/>
+        <v>tc-0.10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>